<commit_message>
alteração do nome da conta r_Despesa_de_Impostos para r_Despesa_IR_CSLL
</commit_message>
<xml_diff>
--- a/V. 2 (Pudim)/dados_teste/DADOS_V2_PUDIM_bp-dreM.xlsx
+++ b/V. 2 (Pudim)/dados_teste/DADOS_V2_PUDIM_bp-dreM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Documents\dev\Finscore\FinScore\V. 2 (Pudim)\dados_teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C25C695-24A2-4764-8BA9-49D2EEDC9532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D841AB7A-4E35-47DE-83F9-EA4BE442803D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="120">
   <si>
     <t>ano</t>
   </si>
@@ -281,9 +281,6 @@
   </si>
   <si>
     <t>r_Resultado_Antes_IR_CSLL − r_Lucro_Liquido</t>
-  </si>
-  <si>
-    <t>r_Despesa_de_Impostos</t>
   </si>
   <si>
     <t>Nomes contábeis mais utilizados</t>
@@ -978,7 +975,7 @@
         <v>19</v>
       </c>
       <c r="U1" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="V1" s="7" t="s">
         <v>17</v>
@@ -28980,13 +28977,13 @@
         <v>28</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C2" s="16" t="s">
         <v>29</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
@@ -28994,7 +28991,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>30</v>
@@ -29008,7 +29005,7 @@
         <v>11</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>21</v>
@@ -29022,7 +29019,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>21</v>
@@ -29036,7 +29033,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C6" s="15" t="s">
         <v>21</v>
@@ -29050,7 +29047,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>21</v>
@@ -29064,7 +29061,7 @@
         <v>16</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>21</v>
@@ -29078,7 +29075,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C9" s="14" t="s">
         <v>36</v>
@@ -29092,7 +29089,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>22</v>
@@ -29106,7 +29103,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>22</v>
@@ -29120,7 +29117,7 @@
         <v>15</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C12" s="15" t="s">
         <v>22</v>
@@ -29134,7 +29131,7 @@
         <v>4</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C13" s="14" t="s">
         <v>35</v>
@@ -29148,7 +29145,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C14" s="15" t="s">
         <v>34</v>
@@ -29162,7 +29159,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C15" s="14" t="s">
         <v>23</v>
@@ -29176,7 +29173,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C16" s="15" t="s">
         <v>23</v>
@@ -29190,7 +29187,7 @@
         <v>5</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>24</v>
@@ -29204,7 +29201,7 @@
         <v>10</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>25</v>
@@ -29218,7 +29215,7 @@
         <v>20</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C19" s="14" t="s">
         <v>25</v>
@@ -29232,7 +29229,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C20" s="15" t="s">
         <v>25</v>
@@ -29246,7 +29243,7 @@
         <v>6</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C21" s="14" t="s">
         <v>25</v>
@@ -29260,7 +29257,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>26</v>
@@ -29271,13 +29268,13 @@
     </row>
     <row r="23" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>32</v>
@@ -29288,7 +29285,7 @@
         <v>17</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>26</v>
@@ -29299,17 +29296,17 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="18" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="18" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="18" t="s">
-        <v>101</v>
-      </c>
-    </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -29336,7 +29333,7 @@
         <v>40</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>41</v>
@@ -29347,7 +29344,7 @@
         <v>42</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C38" s="15" t="s">
         <v>43</v>
@@ -29358,7 +29355,7 @@
         <v>44</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C39" s="15" t="s">
         <v>45</v>
@@ -29369,7 +29366,7 @@
         <v>46</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C40" s="15" t="s">
         <v>47</v>
@@ -29380,7 +29377,7 @@
         <v>48</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C41" s="15" t="s">
         <v>49</v>
@@ -29391,7 +29388,7 @@
         <v>50</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>51</v>
@@ -29402,7 +29399,7 @@
         <v>52</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C43" s="15" t="s">
         <v>53</v>
@@ -29413,7 +29410,7 @@
         <v>54</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>55</v>
@@ -29424,7 +29421,7 @@
         <v>56</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C45" s="15" t="s">
         <v>57</v>
@@ -29435,7 +29432,7 @@
         <v>58</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C46" s="15" t="s">
         <v>59</v>
@@ -29446,7 +29443,7 @@
         <v>60</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C47" s="15" t="s">
         <v>61</v>
@@ -29457,7 +29454,7 @@
         <v>62</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C48" s="15" t="s">
         <v>63</v>
@@ -29468,7 +29465,7 @@
         <v>64</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C49" s="15" t="s">
         <v>65</v>
@@ -29479,7 +29476,7 @@
         <v>66</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C50" s="15" t="s">
         <v>67</v>
@@ -29490,7 +29487,7 @@
         <v>68</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C51" s="15" t="s">
         <v>69</v>
@@ -29501,7 +29498,7 @@
         <v>70</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C52" s="15" t="s">
         <v>71</v>
@@ -29512,7 +29509,7 @@
         <v>72</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C53" s="15" t="s">
         <v>73</v>

</xml_diff>